<commit_message>
First clean deploy of Alex Yap Real Estate
</commit_message>
<xml_diff>
--- a/src/data/communities.xlsx
+++ b/src/data/communities.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\h2oontherock8\Projects\alexyaphomes\src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEBB63F4-22F9-44D0-869A-0E02039E4B1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E05612A3-E66F-46C9-A88F-721D4AF1EC47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="11010" yWindow="2640" windowWidth="26980" windowHeight="17510" xr2:uid="{FE6E1545-603F-4F25-A906-A3DAD4925DF0}"/>
+    <workbookView xWindow="10530" yWindow="3070" windowWidth="26980" windowHeight="17510" xr2:uid="{FE6E1545-603F-4F25-A906-A3DAD4925DF0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="65">
   <si>
     <t>name</t>
   </si>
@@ -48,9 +48,6 @@
     <t>slug</t>
   </si>
   <si>
-    <t>Nestled against the Santa Cruz Mountains, Saratoga offers timeless privacy, premier school districts, and historic hillside acreage.</t>
-  </si>
-  <si>
     <t>A seamless blend of walkable downtown luxury, Michelin-rated dining, and expansive architectural estates tucked along tree-lined foothills.</t>
   </si>
   <si>
@@ -75,9 +72,6 @@
     <t>featured</t>
   </si>
   <si>
-    <t>Featured Order</t>
-  </si>
-  <si>
     <t>Yes</t>
   </si>
   <si>
@@ -190,13 +184,68 @@
   </si>
   <si>
     <t>08 Tree-Lined Avenues &amp; Vibrant Village Warmth</t>
+  </si>
+  <si>
+    <t>https://images.unsplash.com/photo-1628624747186-a941c476b7ef?ixid=M3w4MjcwNjd8MHwxfHNlYXJjaHwyMHx8aG91c2V8ZW58MHx8fHwxNzkyMTc1MjE4fDA&amp;ixlib=rb-4.1.0&amp;w=1200&amp;fit=max&amp;q=80</t>
+  </si>
+  <si>
+    <t>https://images.unsplash.com/photo-1605276374104-dee2a0ed3cd6?ixid=M3w4MjcwNjd8MHwxfHNlYXJjaHwyMnx8aG91c2V8ZW58MHx8fHwxNzkyMTc1MjE4fDA&amp;ixlib=rb-4.1.0&amp;w=1200&amp;fit=max&amp;q=80</t>
+  </si>
+  <si>
+    <t>https://images.unsplash.com/photo-1761013320045-d29e4f10bcbc?ixid=M3w4MjcwNjd8MHwxfHNlYXJjaHwzfHxob21lc3xlbnwwfHx8fDE3OTIxNzU0MzJ8MA&amp;ixlib=rb-4.1.0&amp;w=1200&amp;fit=max&amp;q=80</t>
+  </si>
+  <si>
+    <t>https://images.unsplash.com/photo-1494526585095-c41746248156?ixid=M3w4MjcwNjd8MHwxfHNlYXJjaHwxMHx8aG9tZXN8ZW58MHx8fHwxNzkyMTc1NDMyfDA&amp;ixlib=rb-4.1.0&amp;w=1200&amp;fit=max&amp;q=80</t>
+  </si>
+  <si>
+    <t>https://images.unsplash.com/photo-1777428762767-e3a797da389a?ixid=M3w4MjcwNjd8MHwxfHNlYXJjaHwxNXx8aG9tZXN8ZW58MHx8fHwxNzkyMTc1NDMyfDA&amp;ixlib=rb-4.1.0&amp;w=1200&amp;fit=max&amp;q=80</t>
+  </si>
+  <si>
+    <t>https://images.unsplash.com/photo-1430285561322-7808604715df?ixid=M3w4MjcwNjd8MHwxfHNlYXJjaHwyNnx8aG9tZXN8ZW58MHx8fHwxNzkyMTc1NDMyfDA&amp;ixlib=rb-4.1.0&amp;w=1200&amp;fit=max&amp;q=80</t>
+  </si>
+  <si>
+    <t>featured-order</t>
+  </si>
+  <si>
+    <t>Deciding whether to sell or stay in your home is one of the biggest choices you will make. It takes careful planning to get the highest return on your equity.
+## What It Can Take To Stay Put
+**Important Notice:** Wanting to stay in a home you love makes sense, but most properties require *significant* updates to make single-level living truly functional long-term.
+&gt; "A home gets the highest buyer attention in its first ten days on the market."
+Here are three essential factors to evaluate:
+- Single-story living options and step-free entries
+- Doorway and hallway clearances
+Strategic bathroom modifications
+---
+### Additional Perspectives
+Before making any major renovations, read the latest research from the [Harvard Housing Studies](https://www.jchs.harvard.edu) to see which improvements offer real value.</t>
+  </si>
+  <si>
+    <t>no</t>
+  </si>
+  <si>
+    <t>https://images.unsplash.com/photo-1467385829985-2b0fb82b5193?ixid=M3w4MjcwNjd8MHwxfHNlYXJjaHwxMHx8ZXh0ZXJpb3J8ZW58MHx8fHwxNzkyMTc1MDgxfDA&amp;ixlib=rb-4.1.0&amp;w=1200&amp;fit=max&amp;q=80</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/qogrq7ve/image/upload/v1790284079/cld-sample-4.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/qogrq7ve/image/upload/v1790284067/samples/bike.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/qogrq7ve/image/upload/v1790284066/samples/sheep.jpg</t>
+  </si>
+  <si>
+    <t>https://res.cloudinary.com/qogrq7ve/image/upload/v1790284066/samples/food/pot-mussels.jpg</t>
+  </si>
+  <si>
+    <t>https://images.unsplash.com/photo-1567496898669-ee935f5f647a?ixid=M3w4MjcwNjd8MHwxfHNlYXJjaHwzMHx8aG9tZXN8ZW58MHx8fHwxNzkyMTc1NDMyfDA&amp;ixlib=rb-4.1.0&amp;w=1200&amp;fit=max&amp;q=80</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -235,8 +284,22 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -267,8 +330,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="1"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -291,15 +360,25 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFC4C7C5"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFC4C7C5"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFC4C7C5"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -341,6 +420,15 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -661,352 +749,391 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3A4D0326-1961-46AC-A80E-1EE2BD33E039}">
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:M9"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16" customWidth="1"/>
-    <col min="2" max="2" width="22.90625" customWidth="1"/>
-    <col min="3" max="3" width="45" customWidth="1"/>
-    <col min="4" max="4" width="35.453125" customWidth="1"/>
-    <col min="5" max="9" width="19.453125" customWidth="1"/>
-    <col min="10" max="10" width="19.7265625" customWidth="1"/>
-    <col min="11" max="11" width="18.1796875" customWidth="1"/>
-    <col min="12" max="12" width="15.6328125" customWidth="1"/>
+    <col min="2" max="2" width="16" customWidth="1"/>
+    <col min="3" max="3" width="22.90625" customWidth="1"/>
+    <col min="4" max="4" width="32" customWidth="1"/>
+    <col min="5" max="5" width="35.453125" customWidth="1"/>
+    <col min="6" max="10" width="19.453125" customWidth="1"/>
+    <col min="11" max="11" width="19.7265625" customWidth="1"/>
+    <col min="12" max="12" width="18.1796875" customWidth="1"/>
+    <col min="13" max="13" width="15.6328125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="28" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:13" ht="28" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A1" s="16" t="s">
+        <v>58</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="C1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="F1" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="G1" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="C1" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" s="13" t="s">
+      <c r="H1" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="F1" s="13" t="s">
+      <c r="I1" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="G1" s="13" t="s">
+      <c r="J1" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="H1" s="13" t="s">
+      <c r="K1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="M1" s="15" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" ht="58" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A2" s="2">
+        <f>MAX(A3:A1000) + 1</f>
+        <v>8</v>
+      </c>
+      <c r="B2" s="14" t="s">
         <v>26</v>
       </c>
-      <c r="I1" s="13" t="s">
+      <c r="C2" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="D2" s="6" t="s">
+        <v>42</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>57</v>
+      </c>
+      <c r="F2" s="10" t="s">
+        <v>64</v>
+      </c>
+      <c r="G2" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="H2" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="I2" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="J2" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="K2" s="6" t="str">
+        <f t="shared" ref="K2:K4" si="0">LOWER(SUBSTITUTE(C2, " ", "-"))</f>
+        <v>city-no-01</v>
+      </c>
+      <c r="L2" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="M2" s="2" t="str">
+        <f>IF(L2="YES", COUNTIF(L$2:L2, "YES") &amp; CHOOSE(MIN(COUNTIF(L$2:L2, "YES"), 4), "st", "nd", "rd", "th"), "")</f>
+        <v>1st</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" ht="130" x14ac:dyDescent="0.35">
+      <c r="A3" s="17">
+        <f t="shared" ref="A3:A9" si="1">MAX(A4:A1001) + 1</f>
+        <v>7</v>
+      </c>
+      <c r="B3" s="13" t="s">
         <v>27</v>
       </c>
-      <c r="J1" s="2" t="s">
-        <v>3</v>
-      </c>
-      <c r="K1" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="2" spans="1:12" ht="78" x14ac:dyDescent="0.35">
-      <c r="A2" s="15" t="s">
-        <v>28</v>
-      </c>
-      <c r="B2" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="C2" s="7" t="s">
-        <v>44</v>
-      </c>
-      <c r="D2" s="7" t="s">
+      <c r="C3" s="13" t="s">
+        <v>35</v>
+      </c>
+      <c r="D3" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="E3" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="F2" s="11" t="s">
-        <v>16</v>
-      </c>
-      <c r="G2" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="H2" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="I2" s="11" t="s">
-        <v>18</v>
-      </c>
-      <c r="J2" s="7" t="str">
-        <f t="shared" ref="J2:J9" si="0">LOWER(SUBSTITUTE(B2, " ", "-"))</f>
-        <v>city-no-01</v>
-      </c>
-      <c r="K2" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="L2" s="3" t="str">
-        <f>IF(K2="YES", COUNTIF(K$2:K2, "YES") &amp; CHOOSE(MIN(COUNTIF(K$2:K2, "YES"), 4), "st", "nd", "rd", "th"), "")</f>
-        <v>1st</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" ht="78" x14ac:dyDescent="0.35">
-      <c r="A3" s="14" t="s">
-        <v>29</v>
-      </c>
-      <c r="B3" s="14" t="s">
-        <v>37</v>
-      </c>
-      <c r="C3" s="9" t="s">
-        <v>45</v>
-      </c>
-      <c r="D3" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="E3" s="12" t="s">
-        <v>16</v>
-      </c>
-      <c r="F3" s="12"/>
-      <c r="G3" s="12"/>
-      <c r="H3" s="12"/>
-      <c r="I3" s="12"/>
-      <c r="J3" s="9" t="str">
+      <c r="F3" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="G3" s="11"/>
+      <c r="H3" s="11"/>
+      <c r="I3" s="11"/>
+      <c r="J3" s="11"/>
+      <c r="K3" s="8" t="str">
         <f t="shared" si="0"/>
         <v>city-no-02</v>
       </c>
-      <c r="K3" s="5"/>
-      <c r="L3" s="6" t="str">
-        <f>IF(K3="YES", COUNTIF(K$2:K3, "YES") &amp; CHOOSE(MIN(COUNTIF(K$2:K3, "YES"), 4), "st", "nd", "rd", "th"), "")</f>
+      <c r="L3" s="4"/>
+      <c r="M3" s="5" t="str">
+        <f>IF(L3="YES", COUNTIF(L$2:L3, "YES") &amp; CHOOSE(MIN(COUNTIF(L$2:L3, "YES"), 4), "st", "nd", "rd", "th"), "")</f>
         <v/>
       </c>
     </row>
-    <row r="4" spans="1:12" ht="78" x14ac:dyDescent="0.35">
-      <c r="A4" s="15" t="s">
-        <v>30</v>
-      </c>
-      <c r="B4" s="15" t="s">
-        <v>38</v>
-      </c>
-      <c r="C4" s="7" t="s">
-        <v>46</v>
-      </c>
-      <c r="D4" s="7" t="s">
+    <row r="4" spans="1:13" ht="130" x14ac:dyDescent="0.35">
+      <c r="A4" s="2">
+        <f t="shared" si="1"/>
         <v>6</v>
       </c>
-      <c r="E4" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="F4" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="G4" s="11"/>
-      <c r="H4" s="11"/>
-      <c r="I4" s="11"/>
-      <c r="J4" s="7" t="str">
+      <c r="B4" s="14" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4" s="14" t="s">
+        <v>36</v>
+      </c>
+      <c r="D4" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="E4" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="F4" s="10" t="s">
+        <v>51</v>
+      </c>
+      <c r="G4" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="H4" s="10"/>
+      <c r="I4" s="10"/>
+      <c r="J4" s="10"/>
+      <c r="K4" s="6" t="str">
         <f t="shared" si="0"/>
         <v>city-no-03</v>
       </c>
-      <c r="K4" s="4" t="s">
+      <c r="L4" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="M4" s="2" t="str">
+        <f>IF(L4="YES", COUNTIF(L$2:L4, "YES") &amp; CHOOSE(MIN(COUNTIF(L$2:L4, "YES"), 4), "st", "nd", "rd", "th"), "")</f>
+        <v>2nd</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" ht="143" x14ac:dyDescent="0.35">
+      <c r="A5" s="17">
+        <f t="shared" si="1"/>
+        <v>5</v>
+      </c>
+      <c r="B5" s="13" t="s">
+        <v>29</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="D5" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="E5" s="8" t="s">
+        <v>6</v>
+      </c>
+      <c r="F5" s="11" t="s">
+        <v>59</v>
+      </c>
+      <c r="G5" s="11" t="s">
+        <v>60</v>
+      </c>
+      <c r="H5" s="11" t="s">
+        <v>61</v>
+      </c>
+      <c r="I5" s="11" t="s">
+        <v>62</v>
+      </c>
+      <c r="J5" s="11" t="s">
+        <v>63</v>
+      </c>
+      <c r="K5" s="8" t="str">
+        <f>LOWER(SUBSTITUTE(C5, " ", "-"))</f>
+        <v>city-no-04</v>
+      </c>
+      <c r="L5" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="M5" s="5" t="str">
+        <f>IF(L5="YES", COUNTIF(L$2:L5, "YES") &amp; CHOOSE(MIN(COUNTIF(L$2:L5, "YES"), 4), "st", "nd", "rd", "th"), "")</f>
+        <v>3rd</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" ht="130" x14ac:dyDescent="0.35">
+      <c r="A6" s="2">
+        <f t="shared" si="1"/>
+        <v>4</v>
+      </c>
+      <c r="B6" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C6" s="14" t="s">
+        <v>38</v>
+      </c>
+      <c r="D6" s="6" t="s">
+        <v>46</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>52</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="H6" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="I6" s="7" t="s">
+        <v>19</v>
+      </c>
+      <c r="J6" s="7"/>
+      <c r="K6" s="6" t="str">
+        <f t="shared" ref="K6:K9" si="2">LOWER(SUBSTITUTE(C6, " ", "-"))</f>
+        <v>city-no-05</v>
+      </c>
+      <c r="L6" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="M6" s="2" t="str">
+        <f>IF(L6="YES", COUNTIF(L$2:L6, "YES") &amp; CHOOSE(MIN(COUNTIF(L$2:L6, "YES"), 4), "st", "nd", "rd", "th"), "")</f>
+        <v>4th</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" ht="130" x14ac:dyDescent="0.35">
+      <c r="A7" s="17">
+        <f t="shared" si="1"/>
+        <v>3</v>
+      </c>
+      <c r="B7" s="13" t="s">
+        <v>31</v>
+      </c>
+      <c r="C7" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="D7" s="8" t="s">
+        <v>47</v>
+      </c>
+      <c r="E7" s="8" t="s">
+        <v>8</v>
+      </c>
+      <c r="F7" s="9" t="s">
+        <v>53</v>
+      </c>
+      <c r="G7" s="9" t="s">
+        <v>18</v>
+      </c>
+      <c r="H7" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="I7" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="J7" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="L4" s="3" t="str">
-        <f>IF(K4="YES", COUNTIF(K$2:K4, "YES") &amp; CHOOSE(MIN(COUNTIF(K$2:K4, "YES"), 4), "st", "nd", "rd", "th"), "")</f>
-        <v>2nd</v>
+      <c r="K7" s="8" t="str">
+        <f t="shared" si="2"/>
+        <v>city-no-06</v>
+      </c>
+      <c r="L7" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="M7" s="5" t="str">
+        <f>IF(L7="YES", COUNTIF(L$2:L7, "YES") &amp; CHOOSE(MIN(COUNTIF(L$2:L7, "YES"), 4), "st", "nd", "rd", "th"), "")</f>
+        <v>5th</v>
       </c>
     </row>
-    <row r="5" spans="1:12" ht="78" x14ac:dyDescent="0.35">
-      <c r="A5" s="14" t="s">
-        <v>31</v>
-      </c>
-      <c r="B5" s="14" t="s">
-        <v>39</v>
-      </c>
-      <c r="C5" s="9" t="s">
-        <v>47</v>
-      </c>
-      <c r="D5" s="9" t="s">
-        <v>7</v>
-      </c>
-      <c r="E5" s="12" t="s">
+    <row r="8" spans="1:13" ht="130" x14ac:dyDescent="0.35">
+      <c r="A8" s="2">
+        <f t="shared" si="1"/>
+        <v>2</v>
+      </c>
+      <c r="B8" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C8" s="14" t="s">
+        <v>40</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>9</v>
+      </c>
+      <c r="F8" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="G8" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="H8" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="I8" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="J8" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="F5" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="G5" s="12" t="s">
-        <v>19</v>
-      </c>
-      <c r="H5" s="12"/>
-      <c r="I5" s="12"/>
-      <c r="J5" s="9" t="str">
-        <f>LOWER(SUBSTITUTE(B5, " ", "-"))</f>
-        <v>city-no-04</v>
-      </c>
-      <c r="K5" s="5" t="s">
+      <c r="K8" s="6" t="str">
+        <f t="shared" si="2"/>
+        <v>city-no-07</v>
+      </c>
+      <c r="L8" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="M8" s="2" t="str">
+        <f>IF(L8="YES", COUNTIF(L$2:L8, "YES") &amp; CHOOSE(MIN(COUNTIF(L$2:L8, "YES"), 4), "st", "nd", "rd", "th"), "")</f>
+        <v>6th</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" ht="130" x14ac:dyDescent="0.35">
+      <c r="A9" s="17">
+        <f t="shared" si="1"/>
+        <v>1</v>
+      </c>
+      <c r="B9" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="C9" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>49</v>
+      </c>
+      <c r="E9" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="F9" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="G9" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="H9" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="L5" s="6" t="str">
-        <f>IF(K5="YES", COUNTIF(K$2:K5, "YES") &amp; CHOOSE(MIN(COUNTIF(K$2:K5, "YES"), 4), "st", "nd", "rd", "th"), "")</f>
-        <v>3rd</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" ht="78" x14ac:dyDescent="0.35">
-      <c r="A6" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="B6" s="15" t="s">
-        <v>40</v>
-      </c>
-      <c r="C6" s="7" t="s">
-        <v>48</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>8</v>
-      </c>
-      <c r="E6" s="8" t="s">
-        <v>18</v>
-      </c>
-      <c r="F6" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="G6" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="H6" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="I6" s="8"/>
-      <c r="J6" s="7" t="str">
-        <f t="shared" ref="J6:J9" si="1">LOWER(SUBSTITUTE(B6, " ", "-"))</f>
-        <v>city-no-05</v>
-      </c>
-      <c r="K6" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="L6" s="3" t="str">
-        <f>IF(K6="YES", COUNTIF(K$2:K6, "YES") &amp; CHOOSE(MIN(COUNTIF(K$2:K6, "YES"), 4), "st", "nd", "rd", "th"), "")</f>
-        <v>4th</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" ht="78" x14ac:dyDescent="0.35">
-      <c r="A7" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="B7" s="14" t="s">
-        <v>41</v>
-      </c>
-      <c r="C7" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="D7" s="9" t="s">
-        <v>9</v>
-      </c>
-      <c r="E7" s="10" t="s">
-        <v>19</v>
-      </c>
-      <c r="F7" s="10" t="s">
-        <v>20</v>
-      </c>
-      <c r="G7" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="H7" s="10" t="s">
+      <c r="I9" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="I7" s="10" t="s">
-        <v>16</v>
-      </c>
-      <c r="J7" s="9" t="str">
-        <f t="shared" si="1"/>
-        <v>city-no-06</v>
-      </c>
-      <c r="K7" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="L7" s="6" t="str">
-        <f>IF(K7="YES", COUNTIF(K$2:K7, "YES") &amp; CHOOSE(MIN(COUNTIF(K$2:K7, "YES"), 4), "st", "nd", "rd", "th"), "")</f>
-        <v>5th</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" ht="78" x14ac:dyDescent="0.35">
-      <c r="A8" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="B8" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="C8" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>10</v>
-      </c>
-      <c r="E8" s="11" t="s">
-        <v>20</v>
-      </c>
-      <c r="F8" s="11" t="s">
-        <v>21</v>
-      </c>
-      <c r="G8" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="H8" s="11" t="s">
-        <v>16</v>
-      </c>
-      <c r="I8" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="J8" s="7" t="str">
-        <f t="shared" si="1"/>
-        <v>city-no-07</v>
-      </c>
-      <c r="K8" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="L8" s="3" t="str">
-        <f>IF(K8="YES", COUNTIF(K$2:K8, "YES") &amp; CHOOSE(MIN(COUNTIF(K$2:K8, "YES"), 4), "st", "nd", "rd", "th"), "")</f>
-        <v>6th</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" ht="78" x14ac:dyDescent="0.35">
-      <c r="A9" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="B9" s="14" t="s">
-        <v>43</v>
-      </c>
-      <c r="C9" s="9" t="s">
-        <v>51</v>
-      </c>
-      <c r="D9" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="E9" s="12" t="s">
-        <v>21</v>
-      </c>
-      <c r="F9" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="G9" s="12" t="s">
-        <v>16</v>
-      </c>
-      <c r="H9" s="12" t="s">
-        <v>17</v>
-      </c>
-      <c r="I9" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="J9" s="9" t="str">
-        <f t="shared" si="1"/>
+      <c r="J9" s="11" t="s">
+        <v>13</v>
+      </c>
+      <c r="K9" s="8" t="str">
+        <f t="shared" si="2"/>
         <v>city-no-08</v>
       </c>
-      <c r="K9" s="5" t="s">
-        <v>14</v>
-      </c>
-      <c r="L9" s="6" t="str">
-        <f>IF(K9="YES", COUNTIF(K$2:K9, "YES") &amp; CHOOSE(MIN(COUNTIF(K$2:K9, "YES"), 4), "st", "nd", "rd", "th"), "")</f>
+      <c r="L9" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="M9" s="5" t="str">
+        <f>IF(L9="YES", COUNTIF(L$2:L9, "YES") &amp; CHOOSE(MIN(COUNTIF(L$2:L9, "YES"), 4), "st", "nd", "rd", "th"), "")</f>
         <v>7th</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update property data in excel
</commit_message>
<xml_diff>
--- a/src/data/communities.xlsx
+++ b/src/data/communities.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\h2oontherock8\Projects\alexyaphomes\src\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C55CE2F-35D6-4A31-9ABB-896BC4D12509}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A5E35217-D12E-49D7-9FF0-EBA78FBE5E4D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="6230" yWindow="2360" windowWidth="26980" windowHeight="17510" xr2:uid="{FE6E1545-603F-4F25-A906-A3DAD4925DF0}"/>
+    <workbookView xWindow="9150" yWindow="2820" windowWidth="26980" windowHeight="17510" xr2:uid="{FE6E1545-603F-4F25-A906-A3DAD4925DF0}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,8 +33,30 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="64">
   <si>
     <t>name</t>
   </si>
@@ -112,54 +134,6 @@
   </si>
   <si>
     <t>image-5</t>
-  </si>
-  <si>
-    <t>Community-One</t>
-  </si>
-  <si>
-    <t>Community-Two</t>
-  </si>
-  <si>
-    <t>Community-Three</t>
-  </si>
-  <si>
-    <t>Community-Four</t>
-  </si>
-  <si>
-    <t>Community-Five</t>
-  </si>
-  <si>
-    <t>Community-Six</t>
-  </si>
-  <si>
-    <t>Community-Seven</t>
-  </si>
-  <si>
-    <t>Community-Eight</t>
-  </si>
-  <si>
-    <t>City No-01</t>
-  </si>
-  <si>
-    <t>City No-02</t>
-  </si>
-  <si>
-    <t>City No-03</t>
-  </si>
-  <si>
-    <t>City No-04</t>
-  </si>
-  <si>
-    <t>City No-05</t>
-  </si>
-  <si>
-    <t>City No-06</t>
-  </si>
-  <si>
-    <t>City No-07</t>
-  </si>
-  <si>
-    <t>City No-08</t>
   </si>
   <si>
     <t>01 Distinguished Foothill Estates &amp; Private Vineyards</t>
@@ -240,12 +214,57 @@
   <si>
     <t>https://images.unsplash.com/photo-1567496898669-ee935f5f647a?ixid=M3w4MjcwNjd8MHwxfHNlYXJjaHwzMHx8aG9tZXN8ZW58MHx8fHwxNzkyMTc1NDMyfDA&amp;ixlib=rb-4.1.0&amp;w=1200&amp;fit=max&amp;q=80</t>
   </si>
+  <si>
+    <t>Rivermark</t>
+  </si>
+  <si>
+    <t>Rose Ialand</t>
+  </si>
+  <si>
+    <t>Jungle Island</t>
+  </si>
+  <si>
+    <t>San Jose</t>
+  </si>
+  <si>
+    <t>Mountain View</t>
+  </si>
+  <si>
+    <t>Santa Rosa</t>
+  </si>
+  <si>
+    <t>The Grand Century</t>
+  </si>
+  <si>
+    <t>Complex 6</t>
+  </si>
+  <si>
+    <t>San Francisco</t>
+  </si>
+  <si>
+    <t>Pruneyard Plaza</t>
+  </si>
+  <si>
+    <t>Campbell</t>
+  </si>
+  <si>
+    <t>Terra Serena Luna</t>
+  </si>
+  <si>
+    <t>Milpitas</t>
+  </si>
+  <si>
+    <t>Fish Town</t>
+  </si>
+  <si>
+    <t>Los Altos</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -296,6 +315,12 @@
       <sz val="11"/>
       <color rgb="FFFF0000"/>
       <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF0070C0"/>
+      <name val="Calibri"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -377,7 +402,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -432,6 +457,12 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -758,7 +789,8 @@
     <col min="2" max="2" width="16" customWidth="1"/>
     <col min="3" max="3" width="22.90625" customWidth="1"/>
     <col min="4" max="4" width="32" customWidth="1"/>
-    <col min="5" max="6" width="35.453125" customWidth="1"/>
+    <col min="5" max="5" width="35.453125" customWidth="1"/>
+    <col min="6" max="6" width="32.36328125" customWidth="1"/>
     <col min="7" max="11" width="19.453125" customWidth="1"/>
     <col min="12" max="12" width="19.7265625" customWidth="1"/>
     <col min="13" max="13" width="18.1796875" customWidth="1"/>
@@ -767,7 +799,7 @@
   <sheetData>
     <row r="1" spans="1:14" ht="28" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A1" s="16" t="s">
-        <v>58</v>
+        <v>42</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>0</v>
@@ -806,7 +838,7 @@
         <v>11</v>
       </c>
       <c r="N1" s="15" t="s">
-        <v>56</v>
+        <v>40</v>
       </c>
     </row>
     <row r="2" spans="1:14" ht="58" customHeight="1" x14ac:dyDescent="0.35">
@@ -815,20 +847,23 @@
         <v>8</v>
       </c>
       <c r="B2" s="14" t="s">
+        <v>49</v>
+      </c>
+      <c r="C2" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="D2" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="C2" s="6" t="s">
-        <v>34</v>
-      </c>
-      <c r="D2" s="6" t="s">
-        <v>42</v>
-      </c>
       <c r="E2" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="F2" s="6"/>
+        <v>41</v>
+      </c>
+      <c r="F2" s="19" t="str" cm="1">
+        <f t="array" ref="F2">LOWER(SUBSTITUTE(TRIM(_xlfn.TEXTJOIN("", TRUE, _xlfn.LET(_xlpm.raw, B2 &amp; " " &amp; C2, _xlpm.clean, SUBSTITUTE(SUBSTITUTE(_xlpm.raw, "?", ""), "*", ""), _xlpm.chars, MID(_xlpm.clean, _xlfn.SEQUENCE(LEN(_xlpm.clean)), 1), _xlfn._xlws.FILTER(_xlpm.chars, ISNUMBER(MATCH(_xlpm.chars, {"a","b","c","d","e","f","g","h","i","j","k","l","m","n","o","p","q","r","s","t","u","v","w","x","y","z","A","B","C","D","E","F","G","H","I","J","K","L","M","N","O","P","Q","R","S","T","U","V","W","X","Y","Z","0","1","2","3","4","5","6","7","8","9"," "}, 0)), "")))), " ", "-"))</f>
+        <v>rivermark-san-jose</v>
+      </c>
       <c r="G2" s="10" t="s">
-        <v>64</v>
+        <v>48</v>
       </c>
       <c r="H2" s="10" t="s">
         <v>14</v>
@@ -844,7 +879,7 @@
       </c>
       <c r="L2" s="6" t="str">
         <f t="shared" ref="L2:L4" si="0">LOWER(SUBSTITUTE(C2, " ", "-"))</f>
-        <v>city-no-01</v>
+        <v>san-jose</v>
       </c>
       <c r="M2" s="3" t="s">
         <v>12</v>
@@ -860,20 +895,23 @@
         <v>7</v>
       </c>
       <c r="B3" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="C3" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="D3" s="8" t="s">
         <v>27</v>
-      </c>
-      <c r="C3" s="13" t="s">
-        <v>35</v>
-      </c>
-      <c r="D3" s="8" t="s">
-        <v>43</v>
       </c>
       <c r="E3" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="F3" s="8"/>
+      <c r="F3" s="20" t="str" cm="1">
+        <f t="array" ref="F3">LOWER(SUBSTITUTE(TRIM(_xlfn.TEXTJOIN("", TRUE, _xlfn.LET(_xlpm.raw, B3 &amp; " " &amp; C3, _xlpm.clean, SUBSTITUTE(SUBSTITUTE(_xlpm.raw, "?", ""), "*", ""), _xlpm.chars, MID(_xlpm.clean, _xlfn.SEQUENCE(LEN(_xlpm.clean)), 1), _xlfn._xlws.FILTER(_xlpm.chars, ISNUMBER(MATCH(_xlpm.chars, {"a","b","c","d","e","f","g","h","i","j","k","l","m","n","o","p","q","r","s","t","u","v","w","x","y","z","A","B","C","D","E","F","G","H","I","J","K","L","M","N","O","P","Q","R","S","T","U","V","W","X","Y","Z","0","1","2","3","4","5","6","7","8","9"," "}, 0)), "")))), " ", "-"))</f>
+        <v>rose-ialand-mountain-view</v>
+      </c>
       <c r="G3" s="11" t="s">
-        <v>50</v>
+        <v>34</v>
       </c>
       <c r="H3" s="11"/>
       <c r="I3" s="11"/>
@@ -881,7 +919,7 @@
       <c r="K3" s="11"/>
       <c r="L3" s="8" t="str">
         <f t="shared" si="0"/>
-        <v>city-no-02</v>
+        <v>mountain-view</v>
       </c>
       <c r="M3" s="4"/>
       <c r="N3" s="5" t="str">
@@ -895,20 +933,23 @@
         <v>6</v>
       </c>
       <c r="B4" s="14" t="s">
+        <v>51</v>
+      </c>
+      <c r="C4" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="D4" s="6" t="s">
         <v>28</v>
-      </c>
-      <c r="C4" s="14" t="s">
-        <v>36</v>
-      </c>
-      <c r="D4" s="6" t="s">
-        <v>44</v>
       </c>
       <c r="E4" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="F4" s="6"/>
+      <c r="F4" s="19" t="str" cm="1">
+        <f t="array" ref="F4">LOWER(SUBSTITUTE(TRIM(_xlfn.TEXTJOIN("", TRUE, _xlfn.LET(_xlpm.raw, B4 &amp; " " &amp; C4, _xlpm.clean, SUBSTITUTE(SUBSTITUTE(_xlpm.raw, "?", ""), "*", ""), _xlpm.chars, MID(_xlpm.clean, _xlfn.SEQUENCE(LEN(_xlpm.clean)), 1), _xlfn._xlws.FILTER(_xlpm.chars, ISNUMBER(MATCH(_xlpm.chars, {"a","b","c","d","e","f","g","h","i","j","k","l","m","n","o","p","q","r","s","t","u","v","w","x","y","z","A","B","C","D","E","F","G","H","I","J","K","L","M","N","O","P","Q","R","S","T","U","V","W","X","Y","Z","0","1","2","3","4","5","6","7","8","9"," "}, 0)), "")))), " ", "-"))</f>
+        <v>jungle-island-santa-rosa</v>
+      </c>
       <c r="G4" s="10" t="s">
-        <v>51</v>
+        <v>35</v>
       </c>
       <c r="H4" s="10" t="s">
         <v>13</v>
@@ -918,7 +959,7 @@
       <c r="K4" s="10"/>
       <c r="L4" s="6" t="str">
         <f t="shared" si="0"/>
-        <v>city-no-03</v>
+        <v>santa-rosa</v>
       </c>
       <c r="M4" s="3" t="s">
         <v>12</v>
@@ -934,36 +975,39 @@
         <v>5</v>
       </c>
       <c r="B5" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="D5" s="8" t="s">
         <v>29</v>
-      </c>
-      <c r="C5" s="13" t="s">
-        <v>37</v>
-      </c>
-      <c r="D5" s="8" t="s">
-        <v>45</v>
       </c>
       <c r="E5" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="F5" s="8"/>
+      <c r="F5" s="20" t="str" cm="1">
+        <f t="array" ref="F5">LOWER(SUBSTITUTE(TRIM(_xlfn.TEXTJOIN("", TRUE, _xlfn.LET(_xlpm.raw, B5 &amp; " " &amp; C5, _xlpm.clean, SUBSTITUTE(SUBSTITUTE(_xlpm.raw, "?", ""), "*", ""), _xlpm.chars, MID(_xlpm.clean, _xlfn.SEQUENCE(LEN(_xlpm.clean)), 1), _xlfn._xlws.FILTER(_xlpm.chars, ISNUMBER(MATCH(_xlpm.chars, {"a","b","c","d","e","f","g","h","i","j","k","l","m","n","o","p","q","r","s","t","u","v","w","x","y","z","A","B","C","D","E","F","G","H","I","J","K","L","M","N","O","P","Q","R","S","T","U","V","W","X","Y","Z","0","1","2","3","4","5","6","7","8","9"," "}, 0)), "")))), " ", "-"))</f>
+        <v>the-grand-century-san-jose</v>
+      </c>
       <c r="G5" s="11" t="s">
-        <v>59</v>
+        <v>43</v>
       </c>
       <c r="H5" s="11" t="s">
-        <v>60</v>
+        <v>44</v>
       </c>
       <c r="I5" s="11" t="s">
-        <v>61</v>
+        <v>45</v>
       </c>
       <c r="J5" s="11" t="s">
-        <v>62</v>
+        <v>46</v>
       </c>
       <c r="K5" s="11" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="L5" s="8" t="str">
         <f>LOWER(SUBSTITUTE(C5, " ", "-"))</f>
-        <v>city-no-04</v>
+        <v>san-jose</v>
       </c>
       <c r="M5" s="4" t="s">
         <v>12</v>
@@ -979,20 +1023,23 @@
         <v>4</v>
       </c>
       <c r="B6" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="C6" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="D6" s="6" t="s">
         <v>30</v>
-      </c>
-      <c r="C6" s="14" t="s">
-        <v>38</v>
-      </c>
-      <c r="D6" s="6" t="s">
-        <v>46</v>
       </c>
       <c r="E6" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F6" s="6"/>
+      <c r="F6" s="19" t="str" cm="1">
+        <f t="array" ref="F6">LOWER(SUBSTITUTE(TRIM(_xlfn.TEXTJOIN("", TRUE, _xlfn.LET(_xlpm.raw, B6 &amp; " " &amp; C6, _xlpm.clean, SUBSTITUTE(SUBSTITUTE(_xlpm.raw, "?", ""), "*", ""), _xlpm.chars, MID(_xlpm.clean, _xlfn.SEQUENCE(LEN(_xlpm.clean)), 1), _xlfn._xlws.FILTER(_xlpm.chars, ISNUMBER(MATCH(_xlpm.chars, {"a","b","c","d","e","f","g","h","i","j","k","l","m","n","o","p","q","r","s","t","u","v","w","x","y","z","A","B","C","D","E","F","G","H","I","J","K","L","M","N","O","P","Q","R","S","T","U","V","W","X","Y","Z","0","1","2","3","4","5","6","7","8","9"," "}, 0)), "")))), " ", "-"))</f>
+        <v>complex-6-san-francisco</v>
+      </c>
       <c r="G6" s="7" t="s">
-        <v>52</v>
+        <v>36</v>
       </c>
       <c r="H6" s="7" t="s">
         <v>17</v>
@@ -1006,7 +1053,7 @@
       <c r="K6" s="7"/>
       <c r="L6" s="6" t="str">
         <f t="shared" ref="L6:L9" si="2">LOWER(SUBSTITUTE(C6, " ", "-"))</f>
-        <v>city-no-05</v>
+        <v>san-francisco</v>
       </c>
       <c r="M6" s="3" t="s">
         <v>12</v>
@@ -1022,20 +1069,23 @@
         <v>3</v>
       </c>
       <c r="B7" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="C7" s="13" t="s">
+        <v>59</v>
+      </c>
+      <c r="D7" s="8" t="s">
         <v>31</v>
-      </c>
-      <c r="C7" s="13" t="s">
-        <v>39</v>
-      </c>
-      <c r="D7" s="8" t="s">
-        <v>47</v>
       </c>
       <c r="E7" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="F7" s="8"/>
+      <c r="F7" s="20" t="str" cm="1">
+        <f t="array" ref="F7">LOWER(SUBSTITUTE(TRIM(_xlfn.TEXTJOIN("", TRUE, _xlfn.LET(_xlpm.raw, B7 &amp; " " &amp; C7, _xlpm.clean, SUBSTITUTE(SUBSTITUTE(_xlpm.raw, "?", ""), "*", ""), _xlpm.chars, MID(_xlpm.clean, _xlfn.SEQUENCE(LEN(_xlpm.clean)), 1), _xlfn._xlws.FILTER(_xlpm.chars, ISNUMBER(MATCH(_xlpm.chars, {"a","b","c","d","e","f","g","h","i","j","k","l","m","n","o","p","q","r","s","t","u","v","w","x","y","z","A","B","C","D","E","F","G","H","I","J","K","L","M","N","O","P","Q","R","S","T","U","V","W","X","Y","Z","0","1","2","3","4","5","6","7","8","9"," "}, 0)), "")))), " ", "-"))</f>
+        <v>pruneyard-plaza-campbell</v>
+      </c>
       <c r="G7" s="9" t="s">
-        <v>53</v>
+        <v>37</v>
       </c>
       <c r="H7" s="9" t="s">
         <v>18</v>
@@ -1051,7 +1101,7 @@
       </c>
       <c r="L7" s="8" t="str">
         <f t="shared" si="2"/>
-        <v>city-no-06</v>
+        <v>campbell</v>
       </c>
       <c r="M7" s="4" t="s">
         <v>12</v>
@@ -1067,20 +1117,23 @@
         <v>2</v>
       </c>
       <c r="B8" s="6" t="s">
+        <v>60</v>
+      </c>
+      <c r="C8" s="14" t="s">
+        <v>61</v>
+      </c>
+      <c r="D8" s="6" t="s">
         <v>32</v>
-      </c>
-      <c r="C8" s="14" t="s">
-        <v>40</v>
-      </c>
-      <c r="D8" s="6" t="s">
-        <v>48</v>
       </c>
       <c r="E8" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="F8" s="6"/>
+      <c r="F8" s="19" t="str" cm="1">
+        <f t="array" ref="F8">LOWER(SUBSTITUTE(TRIM(_xlfn.TEXTJOIN("", TRUE, _xlfn.LET(_xlpm.raw, B8 &amp; " " &amp; C8, _xlpm.clean, SUBSTITUTE(SUBSTITUTE(_xlpm.raw, "?", ""), "*", ""), _xlpm.chars, MID(_xlpm.clean, _xlfn.SEQUENCE(LEN(_xlpm.clean)), 1), _xlfn._xlws.FILTER(_xlpm.chars, ISNUMBER(MATCH(_xlpm.chars, {"a","b","c","d","e","f","g","h","i","j","k","l","m","n","o","p","q","r","s","t","u","v","w","x","y","z","A","B","C","D","E","F","G","H","I","J","K","L","M","N","O","P","Q","R","S","T","U","V","W","X","Y","Z","0","1","2","3","4","5","6","7","8","9"," "}, 0)), "")))), " ", "-"))</f>
+        <v>terra-serena-luna-milpitas</v>
+      </c>
       <c r="G8" s="10" t="s">
-        <v>54</v>
+        <v>38</v>
       </c>
       <c r="H8" s="10" t="s">
         <v>19</v>
@@ -1096,7 +1149,7 @@
       </c>
       <c r="L8" s="6" t="str">
         <f t="shared" si="2"/>
-        <v>city-no-07</v>
+        <v>milpitas</v>
       </c>
       <c r="M8" s="3" t="s">
         <v>12</v>
@@ -1112,20 +1165,23 @@
         <v>1</v>
       </c>
       <c r="B9" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="C9" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="D9" s="8" t="s">
         <v>33</v>
-      </c>
-      <c r="C9" s="13" t="s">
-        <v>41</v>
-      </c>
-      <c r="D9" s="8" t="s">
-        <v>49</v>
       </c>
       <c r="E9" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="F9" s="8"/>
+      <c r="F9" s="20" t="str" cm="1">
+        <f t="array" ref="F9">LOWER(SUBSTITUTE(TRIM(_xlfn.TEXTJOIN("", TRUE, _xlfn.LET(_xlpm.raw, B9 &amp; " " &amp; C9, _xlpm.clean, SUBSTITUTE(SUBSTITUTE(_xlpm.raw, "?", ""), "*", ""), _xlpm.chars, MID(_xlpm.clean, _xlfn.SEQUENCE(LEN(_xlpm.clean)), 1), _xlfn._xlws.FILTER(_xlpm.chars, ISNUMBER(MATCH(_xlpm.chars, {"a","b","c","d","e","f","g","h","i","j","k","l","m","n","o","p","q","r","s","t","u","v","w","x","y","z","A","B","C","D","E","F","G","H","I","J","K","L","M","N","O","P","Q","R","S","T","U","V","W","X","Y","Z","0","1","2","3","4","5","6","7","8","9"," "}, 0)), "")))), " ", "-"))</f>
+        <v>fish-town-los-altos</v>
+      </c>
       <c r="G9" s="11" t="s">
-        <v>55</v>
+        <v>39</v>
       </c>
       <c r="H9" s="11" t="s">
         <v>13</v>
@@ -1141,7 +1197,7 @@
       </c>
       <c r="L9" s="8" t="str">
         <f t="shared" si="2"/>
-        <v>city-no-08</v>
+        <v>los-altos</v>
       </c>
       <c r="M9" s="4" t="s">
         <v>12</v>

</xml_diff>